<commit_message>
fix(seed): safely distinguish file contents from disk paths in write_zip_file to prevent Linux OSError Errno 36
</commit_message>
<xml_diff>
--- a/public/chat_files/dennis_old_expense_sheet.xlsx
+++ b/public/chat_files/dennis_old_expense_sheet.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -486,2936 +486,140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="25" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Trip ID</t>
+          <t>Trip Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Truck Registration</t>
+          <t>Truck Reg</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Assigned Driver</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Departure Date</t>
+          <t>Fuel Expense (KES)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Origin Depot</t>
+          <t>Toll Gate</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Destination Facility</t>
+          <t>Driver Allowance</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Cargo Weight (MT)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Diesel Litres</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Fuel Cost (KES)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Fuel Station Location</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Weighbridge Stamp</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Toll &amp; Gate Fees (KES)</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Driver Per Diem (KES)</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>En-Route Repairs (KES)</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Total Trip Expense (KES)</t>
+          <t>Mileage</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TRIP-2026-1001</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>KCU 842P</t>
+          <t>KDC 482B</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Joseph Mutua</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
+          <t>Mombasa to Nairobi</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>42500</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>5000</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>392</v>
-      </c>
-      <c r="I2" s="5" t="n">
-        <v>84084</v>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Shell Mtito Andei Corridor Stop</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8401</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M2" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="5" t="n">
-        <v>94084</v>
+        <v>485</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>TRIP-2026-1002</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>KDA 119M</t>
+          <t>KDD 109F</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Samuel Ochieng</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
+          <t>Nairobi to Eldoret</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>36000</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>4500</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="H3" s="8" t="n">
-        <v>404</v>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>86658</v>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>TotalEnergies Machakos Junction</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8402</t>
-        </is>
-      </c>
-      <c r="L3" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="9" t="n">
-        <v>96658</v>
+        <v>310</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TRIP-2026-1003</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>KDB 482T</t>
+          <t>KDC 482B</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>David Kiprono</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
+          <t>Nairobi to Mombasa</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>41200</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>5000</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>416</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>89232</v>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Rubis Energy Sultan Hamud</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8403</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="5" t="n">
-        <v>99232</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1004</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>KDD 901W</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Francis Mwangi</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>428</v>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>91806</v>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Ola Energy Voi Highway Oasis</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8404</t>
-        </is>
-      </c>
-      <c r="L5" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M5" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N5" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O5" s="9" t="n">
-        <v>104306</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1005</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>KDF 234Q</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Peter Kamau</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>440</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>94380</v>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>National Oil Kibwezi Truck Stop</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8405</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="5" t="n">
-        <v>104380</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1006</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>KCU 842P</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Joseph Mutua</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>452</v>
-      </c>
-      <c r="I7" s="9" t="n">
-        <v>96954</v>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>Shell Mtito Andei Corridor Stop</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8406</t>
-        </is>
-      </c>
-      <c r="L7" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M7" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="9" t="n">
-        <v>106954</v>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1007</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>KDA 119M</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Ochieng</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>464</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>99528</v>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>TotalEnergies Machakos Junction</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8407</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="5" t="n">
-        <v>109528</v>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1008</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>KDB 482T</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>David Kiprono</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>380</v>
-      </c>
-      <c r="I9" s="9" t="n">
-        <v>81510</v>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>Rubis Energy Sultan Hamud</t>
-        </is>
-      </c>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8408</t>
-        </is>
-      </c>
-      <c r="L9" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M9" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N9" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O9" s="9" t="n">
-        <v>94010</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1009</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>KDD 901W</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Francis Mwangi</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>392</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>84084</v>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>Ola Energy Voi Highway Oasis</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8409</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="5" t="n">
-        <v>94084</v>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1010</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>KDF 234Q</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Peter Kamau</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="H11" s="8" t="n">
-        <v>404</v>
-      </c>
-      <c r="I11" s="9" t="n">
-        <v>86658</v>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>National Oil Kibwezi Truck Stop</t>
-        </is>
-      </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8410</t>
-        </is>
-      </c>
-      <c r="L11" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M11" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="9" t="n">
-        <v>96658</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1011</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>KCU 842P</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Joseph Mutua</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>416</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>89232</v>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>Shell Mtito Andei Corridor Stop</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8411</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="5" t="n">
-        <v>99232</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1012</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>KDA 119M</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Samuel Ochieng</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="H13" s="8" t="n">
-        <v>428</v>
-      </c>
-      <c r="I13" s="9" t="n">
-        <v>91806</v>
-      </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>TotalEnergies Machakos Junction</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8412</t>
-        </is>
-      </c>
-      <c r="L13" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M13" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N13" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O13" s="9" t="n">
-        <v>104306</v>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1013</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>KDB 482T</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>David Kiprono</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>440</v>
-      </c>
-      <c r="I14" s="5" t="n">
-        <v>94380</v>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>Rubis Energy Sultan Hamud</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8413</t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="5" t="n">
-        <v>104380</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1014</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>KDD 901W</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Francis Mwangi</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>452</v>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>96954</v>
-      </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>Ola Energy Voi Highway Oasis</t>
-        </is>
-      </c>
-      <c r="K15" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8414</t>
-        </is>
-      </c>
-      <c r="L15" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M15" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="9" t="n">
-        <v>106954</v>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1015</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>KDF 234Q</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Peter Kamau</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>464</v>
-      </c>
-      <c r="I16" s="5" t="n">
-        <v>99528</v>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>National Oil Kibwezi Truck Stop</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8415</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M16" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="5" t="n">
-        <v>109528</v>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1016</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>KCU 842P</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Joseph Mutua</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="H17" s="8" t="n">
-        <v>380</v>
-      </c>
-      <c r="I17" s="9" t="n">
-        <v>81510</v>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t>Shell Mtito Andei Corridor Stop</t>
-        </is>
-      </c>
-      <c r="K17" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8416</t>
-        </is>
-      </c>
-      <c r="L17" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M17" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N17" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O17" s="9" t="n">
-        <v>94010</v>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1017</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>KDA 119M</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Ochieng</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="H18" s="4" t="n">
-        <v>392</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>84084</v>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>TotalEnergies Machakos Junction</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8417</t>
-        </is>
-      </c>
-      <c r="L18" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M18" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="5" t="n">
-        <v>94084</v>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1018</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>KDB 482T</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>David Kiprono</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="H19" s="8" t="n">
-        <v>404</v>
-      </c>
-      <c r="I19" s="9" t="n">
-        <v>86658</v>
-      </c>
-      <c r="J19" s="7" t="inlineStr">
-        <is>
-          <t>Rubis Energy Sultan Hamud</t>
-        </is>
-      </c>
-      <c r="K19" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8418</t>
-        </is>
-      </c>
-      <c r="L19" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M19" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="9" t="n">
-        <v>96658</v>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1019</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>KDD 901W</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Francis Mwangi</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="H20" s="4" t="n">
-        <v>416</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>89232</v>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>Ola Energy Voi Highway Oasis</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8419</t>
-        </is>
-      </c>
-      <c r="L20" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="5" t="n">
-        <v>99232</v>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1020</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>KDF 234Q</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Peter Kamau</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="H21" s="8" t="n">
-        <v>428</v>
-      </c>
-      <c r="I21" s="9" t="n">
-        <v>91806</v>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>National Oil Kibwezi Truck Stop</t>
-        </is>
-      </c>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8420</t>
-        </is>
-      </c>
-      <c r="L21" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M21" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N21" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O21" s="9" t="n">
-        <v>104306</v>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1021</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>KCU 842P</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Joseph Mutua</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>440</v>
-      </c>
-      <c r="I22" s="5" t="n">
-        <v>94380</v>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>Shell Mtito Andei Corridor Stop</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8421</t>
-        </is>
-      </c>
-      <c r="L22" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="5" t="n">
-        <v>104380</v>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1022</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>KDA 119M</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Samuel Ochieng</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="H23" s="8" t="n">
-        <v>452</v>
-      </c>
-      <c r="I23" s="9" t="n">
-        <v>96954</v>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>TotalEnergies Machakos Junction</t>
-        </is>
-      </c>
-      <c r="K23" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8422</t>
-        </is>
-      </c>
-      <c r="L23" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="9" t="n">
-        <v>106954</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1023</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>KDB 482T</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>David Kiprono</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>464</v>
-      </c>
-      <c r="I24" s="5" t="n">
-        <v>99528</v>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>Rubis Energy Sultan Hamud</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8423</t>
-        </is>
-      </c>
-      <c r="L24" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M24" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="5" t="n">
-        <v>109528</v>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1024</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>KDD 901W</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Francis Mwangi</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="H25" s="8" t="n">
-        <v>380</v>
-      </c>
-      <c r="I25" s="9" t="n">
-        <v>81510</v>
-      </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>Ola Energy Voi Highway Oasis</t>
-        </is>
-      </c>
-      <c r="K25" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8424</t>
-        </is>
-      </c>
-      <c r="L25" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M25" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N25" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O25" s="9" t="n">
-        <v>94010</v>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1025</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>KDF 234Q</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Peter Kamau</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="H26" s="4" t="n">
-        <v>392</v>
-      </c>
-      <c r="I26" s="5" t="n">
-        <v>84084</v>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>National Oil Kibwezi Truck Stop</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8425</t>
-        </is>
-      </c>
-      <c r="L26" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M26" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="5" t="n">
-        <v>94084</v>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1026</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>KCU 842P</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Joseph Mutua</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="H27" s="8" t="n">
-        <v>404</v>
-      </c>
-      <c r="I27" s="9" t="n">
-        <v>86658</v>
-      </c>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>Shell Mtito Andei Corridor Stop</t>
-        </is>
-      </c>
-      <c r="K27" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8426</t>
-        </is>
-      </c>
-      <c r="L27" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M27" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N27" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="9" t="n">
-        <v>96658</v>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1027</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>KDA 119M</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Ochieng</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H28" s="4" t="n">
-        <v>416</v>
-      </c>
-      <c r="I28" s="5" t="n">
-        <v>89232</v>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>TotalEnergies Machakos Junction</t>
-        </is>
-      </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8427</t>
-        </is>
-      </c>
-      <c r="L28" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M28" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="5" t="n">
-        <v>99232</v>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1028</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>KDB 482T</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>David Kiprono</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="H29" s="8" t="n">
-        <v>428</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <v>91806</v>
-      </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>Rubis Energy Sultan Hamud</t>
-        </is>
-      </c>
-      <c r="K29" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8428</t>
-        </is>
-      </c>
-      <c r="L29" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M29" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N29" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O29" s="9" t="n">
-        <v>104306</v>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1029</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>KDD 901W</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Francis Mwangi</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="H30" s="4" t="n">
-        <v>440</v>
-      </c>
-      <c r="I30" s="5" t="n">
-        <v>94380</v>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>Ola Energy Voi Highway Oasis</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8429</t>
-        </is>
-      </c>
-      <c r="L30" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M30" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="5" t="n">
-        <v>104380</v>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1030</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>KDF 234Q</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Peter Kamau</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="H31" s="8" t="n">
-        <v>452</v>
-      </c>
-      <c r="I31" s="9" t="n">
-        <v>96954</v>
-      </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>National Oil Kibwezi Truck Stop</t>
-        </is>
-      </c>
-      <c r="K31" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8430</t>
-        </is>
-      </c>
-      <c r="L31" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M31" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N31" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="9" t="n">
-        <v>106954</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1031</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>KCU 842P</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Joseph Mutua</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="H32" s="4" t="n">
-        <v>464</v>
-      </c>
-      <c r="I32" s="5" t="n">
-        <v>99528</v>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>Shell Mtito Andei Corridor Stop</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8431</t>
-        </is>
-      </c>
-      <c r="L32" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M32" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" s="5" t="n">
-        <v>109528</v>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1032</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>KDA 119M</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Samuel Ochieng</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G33" s="8" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="H33" s="8" t="n">
-        <v>380</v>
-      </c>
-      <c r="I33" s="9" t="n">
-        <v>81510</v>
-      </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>TotalEnergies Machakos Junction</t>
-        </is>
-      </c>
-      <c r="K33" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8432</t>
-        </is>
-      </c>
-      <c r="L33" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M33" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N33" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O33" s="9" t="n">
-        <v>94010</v>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1033</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>KDB 482T</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>David Kiprono</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H34" s="4" t="n">
-        <v>392</v>
-      </c>
-      <c r="I34" s="5" t="n">
-        <v>84084</v>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>Rubis Energy Sultan Hamud</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8433</t>
-        </is>
-      </c>
-      <c r="L34" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M34" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" s="5" t="n">
-        <v>94084</v>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1034</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>KDD 901W</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>Francis Mwangi</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G35" s="8" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="H35" s="8" t="n">
-        <v>404</v>
-      </c>
-      <c r="I35" s="9" t="n">
-        <v>86658</v>
-      </c>
-      <c r="J35" s="7" t="inlineStr">
-        <is>
-          <t>Ola Energy Voi Highway Oasis</t>
-        </is>
-      </c>
-      <c r="K35" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8434</t>
-        </is>
-      </c>
-      <c r="L35" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M35" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" s="9" t="n">
-        <v>96658</v>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1035</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>KDF 234Q</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Peter Kamau</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="H36" s="4" t="n">
-        <v>416</v>
-      </c>
-      <c r="I36" s="5" t="n">
-        <v>89232</v>
-      </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>National Oil Kibwezi Truck Stop</t>
-        </is>
-      </c>
-      <c r="K36" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8435</t>
-        </is>
-      </c>
-      <c r="L36" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M36" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" s="5" t="n">
-        <v>99232</v>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1036</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>KCU 842P</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>Joseph Mutua</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G37" s="8" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="H37" s="8" t="n">
-        <v>428</v>
-      </c>
-      <c r="I37" s="9" t="n">
-        <v>91806</v>
-      </c>
-      <c r="J37" s="7" t="inlineStr">
-        <is>
-          <t>Shell Mtito Andei Corridor Stop</t>
-        </is>
-      </c>
-      <c r="K37" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8436</t>
-        </is>
-      </c>
-      <c r="L37" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M37" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N37" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O37" s="9" t="n">
-        <v>104306</v>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1037</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>KDA 119M</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Ochieng</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>440</v>
-      </c>
-      <c r="I38" s="5" t="n">
-        <v>94380</v>
-      </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>TotalEnergies Machakos Junction</t>
-        </is>
-      </c>
-      <c r="K38" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8437</t>
-        </is>
-      </c>
-      <c r="L38" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M38" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" s="5" t="n">
-        <v>104380</v>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1038</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>KDB 482T</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>David Kiprono</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="H39" s="8" t="n">
-        <v>452</v>
-      </c>
-      <c r="I39" s="9" t="n">
-        <v>96954</v>
-      </c>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>Rubis Energy Sultan Hamud</t>
-        </is>
-      </c>
-      <c r="K39" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8438</t>
-        </is>
-      </c>
-      <c r="L39" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M39" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N39" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O39" s="9" t="n">
-        <v>106954</v>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1039</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>KDD 901W</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Francis Mwangi</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H40" s="4" t="n">
-        <v>464</v>
-      </c>
-      <c r="I40" s="5" t="n">
-        <v>99528</v>
-      </c>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t>Ola Energy Voi Highway Oasis</t>
-        </is>
-      </c>
-      <c r="K40" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8439</t>
-        </is>
-      </c>
-      <c r="L40" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M40" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" s="5" t="n">
-        <v>109528</v>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1040</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>KDF 234Q</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>Peter Kamau</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G41" s="8" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="H41" s="8" t="n">
-        <v>380</v>
-      </c>
-      <c r="I41" s="9" t="n">
-        <v>81510</v>
-      </c>
-      <c r="J41" s="7" t="inlineStr">
-        <is>
-          <t>National Oil Kibwezi Truck Stop</t>
-        </is>
-      </c>
-      <c r="K41" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8440</t>
-        </is>
-      </c>
-      <c r="L41" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M41" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N41" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O41" s="9" t="n">
-        <v>94010</v>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1041</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>KCU 842P</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Joseph Mutua</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="H42" s="4" t="n">
-        <v>392</v>
-      </c>
-      <c r="I42" s="5" t="n">
-        <v>84084</v>
-      </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>Shell Mtito Andei Corridor Stop</t>
-        </is>
-      </c>
-      <c r="K42" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8441</t>
-        </is>
-      </c>
-      <c r="L42" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M42" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N42" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O42" s="5" t="n">
-        <v>94084</v>
-      </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1042</t>
-        </is>
-      </c>
-      <c r="B43" s="7" t="inlineStr">
-        <is>
-          <t>KDA 119M</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Samuel Ochieng</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G43" s="8" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="H43" s="8" t="n">
-        <v>404</v>
-      </c>
-      <c r="I43" s="9" t="n">
-        <v>86658</v>
-      </c>
-      <c r="J43" s="7" t="inlineStr">
-        <is>
-          <t>TotalEnergies Machakos Junction</t>
-        </is>
-      </c>
-      <c r="K43" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8442</t>
-        </is>
-      </c>
-      <c r="L43" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M43" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N43" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O43" s="9" t="n">
-        <v>96658</v>
-      </c>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1043</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>KDB 482T</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>David Kiprono</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="H44" s="4" t="n">
-        <v>416</v>
-      </c>
-      <c r="I44" s="5" t="n">
-        <v>89232</v>
-      </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>Rubis Energy Sultan Hamud</t>
-        </is>
-      </c>
-      <c r="K44" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8443</t>
-        </is>
-      </c>
-      <c r="L44" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M44" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N44" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O44" s="5" t="n">
-        <v>99232</v>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1044</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>KDD 901W</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>Francis Mwangi</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>Nairobi Inland Container Depot (ICD)</t>
-        </is>
-      </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>Mombasa Port Berth 19</t>
-        </is>
-      </c>
-      <c r="G45" s="8" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="H45" s="8" t="n">
-        <v>428</v>
-      </c>
-      <c r="I45" s="9" t="n">
-        <v>91806</v>
-      </c>
-      <c r="J45" s="7" t="inlineStr">
-        <is>
-          <t>Ola Energy Voi Highway Oasis</t>
-        </is>
-      </c>
-      <c r="K45" s="7" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8444</t>
-        </is>
-      </c>
-      <c r="L45" s="9" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M45" s="8" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N45" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="O45" s="9" t="n">
-        <v>104306</v>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>TRIP-2026-1045</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>KDF 234Q</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>Peter Kamau</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>Mombasa Port Container Terminal</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>Nairobi ICD Embakasi</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="H46" s="4" t="n">
-        <v>440</v>
-      </c>
-      <c r="I46" s="5" t="n">
-        <v>94380</v>
-      </c>
-      <c r="J46" s="3" t="inlineStr">
-        <is>
-          <t>National Oil Kibwezi Truck Stop</t>
-        </is>
-      </c>
-      <c r="K46" s="3" t="inlineStr">
-        <is>
-          <t>WB-MARIAKANI-8445</t>
-        </is>
-      </c>
-      <c r="L46" s="5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="M46" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O46" s="5" t="n">
-        <v>104380</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
perf: instant in-memory thread switching with pre-seeded recent chats and background loader
</commit_message>
<xml_diff>
--- a/public/chat_files/dennis_old_expense_sheet.xlsx
+++ b/public/chat_files/dennis_old_expense_sheet.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0"/>
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -486,140 +486,2936 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Trip Date</t>
+          <t>Trip ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Truck Reg</t>
+          <t>Truck Registration</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Assigned Driver</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Fuel Expense (KES)</t>
+          <t>Departure Date</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Toll Gate</t>
+          <t>Origin Depot</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Driver Allowance</t>
+          <t>Destination Facility</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Mileage</t>
+          <t>Cargo Weight (MT)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Diesel Litres</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Fuel Cost (KES)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Fuel Station Location</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Weighbridge Stamp</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Toll &amp; Gate Fees (KES)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Driver Per Diem (KES)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>En-Route Repairs (KES)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Total Trip Expense (KES)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>TRIP-2026-1001</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>KDC 482B</t>
+          <t>KCU 842P</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Mombasa to Nairobi</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>42500</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>3200</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>5000</v>
+          <t>Joseph Mutua</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>485</v>
+        <v>26</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>392</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>84084</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Shell Mtito Andei Corridor Stop</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8401</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="5" t="n">
+        <v>94084</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>TRIP-2026-1002</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>KDD 109F</t>
+          <t>KDA 119M</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Nairobi to Eldoret</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="n">
-        <v>36000</v>
-      </c>
-      <c r="E3" s="9" t="n">
-        <v>1800</v>
-      </c>
-      <c r="F3" s="9" t="n">
-        <v>4500</v>
+          <t>Samuel Ochieng</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
       </c>
       <c r="G3" s="8" t="n">
-        <v>310</v>
+        <v>27.5</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>404</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>86658</v>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>TotalEnergies Machakos Junction</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8402</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="9" t="n">
+        <v>96658</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>TRIP-2026-1003</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>KDC 482B</t>
+          <t>KDB 482T</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Nairobi to Mombasa</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>41200</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>3200</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>5000</v>
+          <t>David Kiprono</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>485</v>
+        <v>29</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>416</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>89232</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Rubis Energy Sultan Hamud</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8403</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="5" t="n">
+        <v>99232</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1004</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>KDD 901W</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Francis Mwangi</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>428</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>91806</v>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Ola Energy Voi Highway Oasis</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8404</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M5" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O5" s="9" t="n">
+        <v>104306</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>KDF 234Q</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Peter Kamau</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>94380</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>National Oil Kibwezi Truck Stop</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8405</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="5" t="n">
+        <v>104380</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1006</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>KCU 842P</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Joseph Mutua</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>452</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>96954</v>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Shell Mtito Andei Corridor Stop</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8406</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M7" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="9" t="n">
+        <v>106954</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>KDA 119M</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Ochieng</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>464</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>99528</v>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>TotalEnergies Machakos Junction</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8407</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="5" t="n">
+        <v>109528</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1008</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>KDB 482T</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>David Kiprono</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>81510</v>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Rubis Energy Sultan Hamud</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8408</t>
+        </is>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M9" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O9" s="9" t="n">
+        <v>94010</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>KDD 901W</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Francis Mwangi</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>392</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>84084</v>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Ola Energy Voi Highway Oasis</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8409</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="5" t="n">
+        <v>94084</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1010</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>KDF 234Q</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Peter Kamau</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>404</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>86658</v>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>National Oil Kibwezi Truck Stop</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8410</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="9" t="n">
+        <v>96658</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>KCU 842P</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Joseph Mutua</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>416</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>89232</v>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Shell Mtito Andei Corridor Stop</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8411</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="5" t="n">
+        <v>99232</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1012</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>KDA 119M</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Samuel Ochieng</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>428</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>91806</v>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>TotalEnergies Machakos Junction</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8412</t>
+        </is>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M13" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O13" s="9" t="n">
+        <v>104306</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>KDB 482T</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>David Kiprono</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>94380</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Rubis Energy Sultan Hamud</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8413</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="5" t="n">
+        <v>104380</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1014</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>KDD 901W</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Francis Mwangi</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>452</v>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>96954</v>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Ola Energy Voi Highway Oasis</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8414</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M15" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="9" t="n">
+        <v>106954</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1015</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>KDF 234Q</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Peter Kamau</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>464</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>99528</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>National Oil Kibwezi Truck Stop</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8415</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="5" t="n">
+        <v>109528</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1016</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>KCU 842P</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Joseph Mutua</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>81510</v>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>Shell Mtito Andei Corridor Stop</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8416</t>
+        </is>
+      </c>
+      <c r="L17" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M17" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O17" s="9" t="n">
+        <v>94010</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>KDA 119M</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Ochieng</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>392</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>84084</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>TotalEnergies Machakos Junction</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8417</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="5" t="n">
+        <v>94084</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1018</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>KDB 482T</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>David Kiprono</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>404</v>
+      </c>
+      <c r="I19" s="9" t="n">
+        <v>86658</v>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>Rubis Energy Sultan Hamud</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8418</t>
+        </is>
+      </c>
+      <c r="L19" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="9" t="n">
+        <v>96658</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1019</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>KDD 901W</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Francis Mwangi</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>416</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>89232</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Ola Energy Voi Highway Oasis</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8419</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="5" t="n">
+        <v>99232</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1020</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>KDF 234Q</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Peter Kamau</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>428</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>91806</v>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>National Oil Kibwezi Truck Stop</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8420</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M21" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N21" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O21" s="9" t="n">
+        <v>104306</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1021</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>KCU 842P</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Joseph Mutua</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>94380</v>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Shell Mtito Andei Corridor Stop</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8421</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="5" t="n">
+        <v>104380</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1022</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>KDA 119M</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Samuel Ochieng</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>452</v>
+      </c>
+      <c r="I23" s="9" t="n">
+        <v>96954</v>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>TotalEnergies Machakos Junction</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8422</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="9" t="n">
+        <v>106954</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1023</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>KDB 482T</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>David Kiprono</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>464</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>99528</v>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Rubis Energy Sultan Hamud</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8423</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="5" t="n">
+        <v>109528</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1024</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>KDD 901W</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Francis Mwangi</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>81510</v>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>Ola Energy Voi Highway Oasis</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8424</t>
+        </is>
+      </c>
+      <c r="L25" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M25" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N25" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O25" s="9" t="n">
+        <v>94010</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1025</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>KDF 234Q</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Peter Kamau</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>392</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>84084</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>National Oil Kibwezi Truck Stop</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8425</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="5" t="n">
+        <v>94084</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1026</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>KCU 842P</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Joseph Mutua</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>404</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>86658</v>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>Shell Mtito Andei Corridor Stop</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8426</t>
+        </is>
+      </c>
+      <c r="L27" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M27" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="9" t="n">
+        <v>96658</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1027</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>KDA 119M</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Ochieng</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>416</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>89232</v>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>TotalEnergies Machakos Junction</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8427</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="5" t="n">
+        <v>99232</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1028</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>KDB 482T</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>David Kiprono</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>428</v>
+      </c>
+      <c r="I29" s="9" t="n">
+        <v>91806</v>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>Rubis Energy Sultan Hamud</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8428</t>
+        </is>
+      </c>
+      <c r="L29" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N29" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O29" s="9" t="n">
+        <v>104306</v>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1029</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>KDD 901W</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Francis Mwangi</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>94380</v>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Ola Energy Voi Highway Oasis</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8429</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="5" t="n">
+        <v>104380</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1030</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>KDF 234Q</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Peter Kamau</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H31" s="8" t="n">
+        <v>452</v>
+      </c>
+      <c r="I31" s="9" t="n">
+        <v>96954</v>
+      </c>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>National Oil Kibwezi Truck Stop</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8430</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M31" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N31" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="9" t="n">
+        <v>106954</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1031</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>KCU 842P</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Joseph Mutua</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>464</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>99528</v>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Shell Mtito Andei Corridor Stop</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8431</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="5" t="n">
+        <v>109528</v>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1032</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>KDA 119M</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Samuel Ochieng</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="I33" s="9" t="n">
+        <v>81510</v>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>TotalEnergies Machakos Junction</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8432</t>
+        </is>
+      </c>
+      <c r="L33" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M33" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N33" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O33" s="9" t="n">
+        <v>94010</v>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1033</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>KDB 482T</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>David Kiprono</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>392</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>84084</v>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Rubis Energy Sultan Hamud</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8433</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M34" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="5" t="n">
+        <v>94084</v>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1034</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>KDD 901W</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Francis Mwangi</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>404</v>
+      </c>
+      <c r="I35" s="9" t="n">
+        <v>86658</v>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>Ola Energy Voi Highway Oasis</t>
+        </is>
+      </c>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8434</t>
+        </is>
+      </c>
+      <c r="L35" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="9" t="n">
+        <v>96658</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1035</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>KDF 234Q</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Peter Kamau</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>416</v>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>89232</v>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>National Oil Kibwezi Truck Stop</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8435</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="5" t="n">
+        <v>99232</v>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1036</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>KCU 842P</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Joseph Mutua</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>428</v>
+      </c>
+      <c r="I37" s="9" t="n">
+        <v>91806</v>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>Shell Mtito Andei Corridor Stop</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8436</t>
+        </is>
+      </c>
+      <c r="L37" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M37" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N37" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O37" s="9" t="n">
+        <v>104306</v>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1037</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>KDA 119M</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Ochieng</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>94380</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>TotalEnergies Machakos Junction</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8437</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M38" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="5" t="n">
+        <v>104380</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1038</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>KDB 482T</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>David Kiprono</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H39" s="8" t="n">
+        <v>452</v>
+      </c>
+      <c r="I39" s="9" t="n">
+        <v>96954</v>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>Rubis Energy Sultan Hamud</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8438</t>
+        </is>
+      </c>
+      <c r="L39" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M39" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N39" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="9" t="n">
+        <v>106954</v>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1039</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>KDD 901W</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Francis Mwangi</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>464</v>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>99528</v>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Ola Energy Voi Highway Oasis</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8439</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="5" t="n">
+        <v>109528</v>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1040</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>KDF 234Q</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Peter Kamau</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="H41" s="8" t="n">
+        <v>380</v>
+      </c>
+      <c r="I41" s="9" t="n">
+        <v>81510</v>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>National Oil Kibwezi Truck Stop</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8440</t>
+        </is>
+      </c>
+      <c r="L41" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M41" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N41" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O41" s="9" t="n">
+        <v>94010</v>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1041</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>KCU 842P</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Joseph Mutua</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>392</v>
+      </c>
+      <c r="I42" s="5" t="n">
+        <v>84084</v>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Shell Mtito Andei Corridor Stop</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8441</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M42" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="5" t="n">
+        <v>94084</v>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1042</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>KDA 119M</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Samuel Ochieng</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H43" s="8" t="n">
+        <v>404</v>
+      </c>
+      <c r="I43" s="9" t="n">
+        <v>86658</v>
+      </c>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>TotalEnergies Machakos Junction</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8442</t>
+        </is>
+      </c>
+      <c r="L43" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M43" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="9" t="n">
+        <v>96658</v>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1043</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>KDB 482T</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>David Kiprono</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>416</v>
+      </c>
+      <c r="I44" s="5" t="n">
+        <v>89232</v>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Rubis Energy Sultan Hamud</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8443</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M44" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="5" t="n">
+        <v>99232</v>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1044</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>KDD 901W</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Francis Mwangi</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Nairobi Inland Container Depot (ICD)</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Mombasa Port Berth 19</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H45" s="8" t="n">
+        <v>428</v>
+      </c>
+      <c r="I45" s="9" t="n">
+        <v>91806</v>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>Ola Energy Voi Highway Oasis</t>
+        </is>
+      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8444</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M45" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N45" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O45" s="9" t="n">
+        <v>104306</v>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>TRIP-2026-1045</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>KDF 234Q</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Peter Kamau</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Mombasa Port Container Terminal</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Nairobi ICD Embakasi</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="I46" s="5" t="n">
+        <v>94380</v>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>National Oil Kibwezi Truck Stop</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>WB-MARIAKANI-8445</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="M46" s="4" t="n">
+        <v>6500</v>
+      </c>
+      <c r="N46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="5" t="n">
+        <v>104380</v>
       </c>
     </row>
   </sheetData>

</xml_diff>